<commit_message>
feat: melhorias no frontend (mapa escuro, banner offline, otimizacao tatil) e backend (rate limiting, excecoes http, webhook signature) e atualizacao do README
</commit_message>
<xml_diff>
--- a/01-08-2026 MATEUS CARMOZINO DE OLIVEIRA.xlsx
+++ b/01-08-2026 MATEUS CARMOZINO DE OLIVEIRA.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37CF3885-2E07-409F-AC0D-B34662B5B30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F4E52C-D6F7-4F0A-AC78-B1D93AE3757A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1144,6 +1144,7 @@
   <dimension ref="A1:J85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
     <col min="7" max="7" width="9.5546875" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>

</xml_diff>